<commit_message>
fix(CORE-000206): correct Match Datasets keys and test data
Match Datasets entries used IDVAR/IDVARVAL as literal join keys, which
the Child:true SQL merge treats as column names, causing every dataset
to error with "Column idvar not found". Drop IDVAR/IDVARVAL from Keys
so the LEFT JOIN brings in parent columns for value_is_reference to
resolve dynamically. Also add missing IDVAR/IDVARVAL columns to the
positive/02 test data, fix a typo in the Outcome message, and rebuild
the negative test Validation sheet/highlights to match real engine
errors.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/CORE-000206/negative/01/data/unit-test-coreid-CG0371-negative.xlsx
+++ b/rules/CORE-000206/negative/01/data/unit-test-coreid-CG0371-negative.xlsx
@@ -1,11 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
@@ -17,33 +13,38 @@
     <sheet name="lb.xpt" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color indexed="8"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -56,17 +57,15 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -75,104 +74,31 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="6"/>
-      </left>
-      <right style="thin">
-        <color theme="6"/>
-      </right>
-      <top style="thin">
-        <color theme="6"/>
-      </top>
-      <bottom style="medium">
-        <color theme="6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -319,6 +245,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -353,6 +280,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -387,20 +315,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -522,7 +446,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -537,12 +500,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
@@ -575,12 +538,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Filename</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
@@ -657,38 +620,486 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Error group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Error level</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Row num</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>supplb.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RDOMAIN</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>supplb.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>supplb.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>IDVAR</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LBSEQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>supplb.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IDVARVAL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>RDOMAIN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>IDVAR</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LBSEQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>IDVARVAL</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>RDOMAIN</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>IDVAR</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>AESEQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>relrec.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>IDVARVAL</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>co.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>RDOMAIN</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>co.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>co.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>IDVAR</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>LBGRPID</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>co.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>IDVARVAL</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
     </row>
@@ -707,235 +1118,235 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>RDOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>IDVAR</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>IDVARVAL</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>QNAM</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>QLABEL</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>QVAL</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>QORIG</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>QEVAL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Related Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable Value</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Qualifier Variable Name</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Qualifier Variable Label</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Data Value</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Evaluator</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="3" t="n">
+      <c r="A4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="4" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>LB</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>LBSEQ</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>LBCLSIG</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Clinically Significant</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>CRF</t>
         </is>
@@ -956,208 +1367,208 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>RDOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>IDVAR</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>IDVARVAL</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>RELTYPE</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>RELID</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Related Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable Value</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Relationship Type</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Relationship Identifier</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3" t="n">
+      <c r="A4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>LB</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>LBSEQ</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>ONE</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>AE</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>AESEQ</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>ONE</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -1178,284 +1589,284 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>RDOMAIN</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>COSEQ</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>IDVAR</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>IDVARVAL</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>COREF</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>COVAL</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>COEVAL</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>COEVALID</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>CODTC</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>CODY</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Related Domain Abbreviation</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Identifying Variable Value</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Comment Reference</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Evaluator</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Evaluator Identifier</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Date/Time of Comment</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Study Day of Comment</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="E4" s="3" t="n">
+      <c r="A4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="3" t="n">
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>CO</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>LB</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>LBGRPID</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>test comment</t>
         </is>
@@ -1476,169 +1887,169 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>AESEQ</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>AETERM</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>AEDECOD</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>AESTDTC</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Reported Term for the Adverse Event</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Standardized Disposition Term</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Start Date/Time of Adverse Event</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="7" t="n">
+      <c r="A4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="F4" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="7" t="n">
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>AE</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>AE1</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>AE1</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>2021-02-26</t>
         </is>
@@ -1659,1186 +2070,1186 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>STUDYID</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DOMAIN</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>LBSEQ</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>LBGRPID</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>LBREFID</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>LBSPID</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>LBTESTCD</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>LBTEST</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>LBTSTCND</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>LBBDAGNT</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>LBTSTOPO</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>LBCAT</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>LBSCAT</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>LBORRES</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>LBORRESU</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>LBRESSCL</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>LBRESTYP</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>LBCOLSRT</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>LBORNRLO</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>LBORNRHI</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>LBLLOD</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>LBSTRESC</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>LBSTRESN</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>LBSTRESU</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>LBSTNRLO</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>LBSTNRHI</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>LBSTNRC</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>LBNRIND</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>LBSTAT</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AE1" s="3" t="inlineStr">
         <is>
           <t>LBREASND</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>LBNAM</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AG1" s="3" t="inlineStr">
         <is>
           <t>LBLOINC</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>LBSPEC</t>
         </is>
       </c>
-      <c r="AI1" s="2" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>LBSPCCND</t>
         </is>
       </c>
-      <c r="AJ1" s="2" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>LBSPCUFL</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>LBMETHOD</t>
         </is>
       </c>
-      <c r="AL1" s="2" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
         <is>
           <t>LBANMETH</t>
         </is>
       </c>
-      <c r="AM1" s="2" t="inlineStr">
+      <c r="AM1" s="3" t="inlineStr">
         <is>
           <t>LBTMTHSN</t>
         </is>
       </c>
-      <c r="AN1" s="2" t="inlineStr">
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>LBLOBXFL</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="AO1" s="3" t="inlineStr">
         <is>
           <t>LBBLFL</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
+      <c r="AP1" s="3" t="inlineStr">
         <is>
           <t>LBFAST</t>
         </is>
       </c>
-      <c r="AQ1" s="2" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>LBDRVFL</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>LBTOX</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>LBTOXGR</t>
         </is>
       </c>
-      <c r="AT1" s="2" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>LBCLSIG</t>
         </is>
       </c>
-      <c r="AU1" s="2" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>VISITNUM</t>
         </is>
       </c>
-      <c r="AV1" s="2" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>VISIT</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>VISITDY</t>
         </is>
       </c>
-      <c r="AX1" s="2" t="inlineStr">
+      <c r="AX1" s="3" t="inlineStr">
         <is>
           <t>TAETORD</t>
         </is>
       </c>
-      <c r="AY1" s="2" t="inlineStr">
+      <c r="AY1" s="3" t="inlineStr">
         <is>
           <t>EPOCH</t>
         </is>
       </c>
-      <c r="AZ1" s="2" t="inlineStr">
+      <c r="AZ1" s="3" t="inlineStr">
         <is>
           <t>LBDTC</t>
         </is>
       </c>
-      <c r="BA1" s="2" t="inlineStr">
+      <c r="BA1" s="3" t="inlineStr">
         <is>
           <t>LBENDTC</t>
         </is>
       </c>
-      <c r="BB1" s="2" t="inlineStr">
+      <c r="BB1" s="3" t="inlineStr">
         <is>
           <t>LBDY</t>
         </is>
       </c>
-      <c r="BC1" s="2" t="inlineStr">
+      <c r="BC1" s="3" t="inlineStr">
         <is>
           <t>LBENDY</t>
         </is>
       </c>
-      <c r="BD1" s="2" t="inlineStr">
+      <c r="BD1" s="3" t="inlineStr">
         <is>
           <t>LBTPT</t>
         </is>
       </c>
-      <c r="BE1" s="2" t="inlineStr">
+      <c r="BE1" s="3" t="inlineStr">
         <is>
           <t>LBTPTNUM</t>
         </is>
       </c>
-      <c r="BF1" s="2" t="inlineStr">
+      <c r="BF1" s="3" t="inlineStr">
         <is>
           <t>LBELTM</t>
         </is>
       </c>
-      <c r="BG1" s="2" t="inlineStr">
+      <c r="BG1" s="3" t="inlineStr">
         <is>
           <t>LBTPTREF</t>
         </is>
       </c>
-      <c r="BH1" s="2" t="inlineStr">
+      <c r="BH1" s="3" t="inlineStr">
         <is>
           <t>LBRFTDTC</t>
         </is>
       </c>
-      <c r="BI1" s="2" t="inlineStr">
+      <c r="BI1" s="3" t="inlineStr">
         <is>
           <t>LBPTFL</t>
         </is>
       </c>
-      <c r="BJ1" s="2" t="inlineStr">
+      <c r="BJ1" s="3" t="inlineStr">
         <is>
           <t>LBPDUR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Study Identifier</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Domain Abbreviation</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Unique Subject Identifier</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Sequence Number</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Group ID</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Specimen ID</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Sponsor-Defined Identifier</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Lab Test or Examination Short Name</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Lab Test or Examination Name</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Test Condition</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Binding Agent</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Test Operational Objective</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Category for Lab Test</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>Subcategory for Lab Test</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Result or Finding in Original Units</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Original Units</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>Result Scale</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>Result Type</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Collected Summary Result Type</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>Reference Range Lower Limit in Orig Unit</t>
         </is>
       </c>
-      <c r="U2" s="3" t="inlineStr">
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>Reference Range Upper Limit in Orig Unit</t>
         </is>
       </c>
-      <c r="V2" s="3" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>Lower Limit of Detection</t>
         </is>
       </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="W2" s="4" t="inlineStr">
         <is>
           <t>Character Result/Finding in Std Format</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>Numeric Result/Finding in Standard Units</t>
         </is>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>Standard Units</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>Reference Range Lower Limit-Std Units</t>
         </is>
       </c>
-      <c r="AA2" s="3" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>Reference Range Upper Limit-Std Units</t>
         </is>
       </c>
-      <c r="AB2" s="3" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>Reference Range for Char Rslt-Std Units</t>
         </is>
       </c>
-      <c r="AC2" s="3" t="inlineStr">
+      <c r="AC2" s="4" t="inlineStr">
         <is>
           <t>Reference Range Indicator</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="inlineStr">
+      <c r="AD2" s="4" t="inlineStr">
         <is>
           <t>Completion Status</t>
         </is>
       </c>
-      <c r="AE2" s="3" t="inlineStr">
+      <c r="AE2" s="4" t="inlineStr">
         <is>
           <t>Reason Test Not Done</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
+      <c r="AF2" s="4" t="inlineStr">
         <is>
           <t>Vendor Name</t>
         </is>
       </c>
-      <c r="AG2" s="3" t="inlineStr">
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>LOINC Code</t>
         </is>
       </c>
-      <c r="AH2" s="3" t="inlineStr">
+      <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>Specimen Type</t>
         </is>
       </c>
-      <c r="AI2" s="3" t="inlineStr">
+      <c r="AI2" s="4" t="inlineStr">
         <is>
           <t>Specimen Condition</t>
         </is>
       </c>
-      <c r="AJ2" s="3" t="inlineStr">
+      <c r="AJ2" s="4" t="inlineStr">
         <is>
           <t>Specimen Usability for the Test</t>
         </is>
       </c>
-      <c r="AK2" s="3" t="inlineStr">
+      <c r="AK2" s="4" t="inlineStr">
         <is>
           <t>Method of Test or Examination</t>
         </is>
       </c>
-      <c r="AL2" s="3" t="inlineStr">
+      <c r="AL2" s="4" t="inlineStr">
         <is>
           <t>Analysis Method</t>
         </is>
       </c>
-      <c r="AM2" s="3" t="inlineStr">
+      <c r="AM2" s="4" t="inlineStr">
         <is>
           <t>Test Method Sensitivity</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="inlineStr">
+      <c r="AN2" s="4" t="inlineStr">
         <is>
           <t>Last Observation Before Exposure Flag</t>
         </is>
       </c>
-      <c r="AO2" s="3" t="inlineStr">
+      <c r="AO2" s="4" t="inlineStr">
         <is>
           <t>Baseline Flag</t>
         </is>
       </c>
-      <c r="AP2" s="3" t="inlineStr">
+      <c r="AP2" s="4" t="inlineStr">
         <is>
           <t>Fasting Status</t>
         </is>
       </c>
-      <c r="AQ2" s="3" t="inlineStr">
+      <c r="AQ2" s="4" t="inlineStr">
         <is>
           <t>Derived Flag</t>
         </is>
       </c>
-      <c r="AR2" s="3" t="inlineStr">
+      <c r="AR2" s="4" t="inlineStr">
         <is>
           <t>Toxicity</t>
         </is>
       </c>
-      <c r="AS2" s="3" t="inlineStr">
+      <c r="AS2" s="4" t="inlineStr">
         <is>
           <t>Standard Toxicity Grade</t>
         </is>
       </c>
-      <c r="AT2" s="3" t="inlineStr">
+      <c r="AT2" s="4" t="inlineStr">
         <is>
           <t>Clinically Significant, Collected</t>
         </is>
       </c>
-      <c r="AU2" s="3" t="inlineStr">
+      <c r="AU2" s="4" t="inlineStr">
         <is>
           <t>Visit Number</t>
         </is>
       </c>
-      <c r="AV2" s="3" t="inlineStr">
+      <c r="AV2" s="4" t="inlineStr">
         <is>
           <t>Visit Name</t>
         </is>
       </c>
-      <c r="AW2" s="3" t="inlineStr">
+      <c r="AW2" s="4" t="inlineStr">
         <is>
           <t>Planned Study Day of Visit</t>
         </is>
       </c>
-      <c r="AX2" s="3" t="inlineStr">
+      <c r="AX2" s="4" t="inlineStr">
         <is>
           <t>Planned Order of Element within Arm</t>
         </is>
       </c>
-      <c r="AY2" s="3" t="inlineStr">
+      <c r="AY2" s="4" t="inlineStr">
         <is>
           <t>Epoch</t>
         </is>
       </c>
-      <c r="AZ2" s="3" t="inlineStr">
+      <c r="AZ2" s="4" t="inlineStr">
         <is>
           <t>Date/Time of Specimen Collection</t>
         </is>
       </c>
-      <c r="BA2" s="3" t="inlineStr">
+      <c r="BA2" s="4" t="inlineStr">
         <is>
           <t>End Date/Time of Specimen Collection</t>
         </is>
       </c>
-      <c r="BB2" s="3" t="inlineStr">
+      <c r="BB2" s="4" t="inlineStr">
         <is>
           <t>Study Day of Specimen Collection</t>
         </is>
       </c>
-      <c r="BC2" s="3" t="inlineStr">
+      <c r="BC2" s="4" t="inlineStr">
         <is>
           <t>Study Day of End of Observation</t>
         </is>
       </c>
-      <c r="BD2" s="3" t="inlineStr">
+      <c r="BD2" s="4" t="inlineStr">
         <is>
           <t>Planned Time Point Name</t>
         </is>
       </c>
-      <c r="BE2" s="3" t="inlineStr">
+      <c r="BE2" s="4" t="inlineStr">
         <is>
           <t>Planned Time Point Number</t>
         </is>
       </c>
-      <c r="BF2" s="3" t="inlineStr">
+      <c r="BF2" s="4" t="inlineStr">
         <is>
           <t>Planned Elapsed Time from Time Point Ref</t>
         </is>
       </c>
-      <c r="BG2" s="3" t="inlineStr">
+      <c r="BG2" s="4" t="inlineStr">
         <is>
           <t>Time Point Reference</t>
         </is>
       </c>
-      <c r="BH2" s="3" t="inlineStr">
+      <c r="BH2" s="4" t="inlineStr">
         <is>
           <t>Date/Time of Reference Time Point</t>
         </is>
       </c>
-      <c r="BI2" s="3" t="inlineStr">
+      <c r="BI2" s="4" t="inlineStr">
         <is>
           <t>Point in Time Flag</t>
         </is>
       </c>
-      <c r="BJ2" s="3" t="inlineStr">
+      <c r="BJ2" s="4" t="inlineStr">
         <is>
           <t>Planned Duration</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="U3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="V3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="W3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="X3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="W3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="X3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="Z3" s="3" t="inlineStr">
+      <c r="Y3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="Z3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AA3" s="3" t="inlineStr">
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AB3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AC3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AD3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AE3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AF3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AG3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AH3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AI3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AJ3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AK3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AL3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AM3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AN3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AO3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AP3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AQ3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AR3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AS3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AT3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AU3" s="3" t="inlineStr">
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AC3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AD3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AE3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AF3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AG3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AH3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AI3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AK3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AL3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AM3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AN3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AO3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AP3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AQ3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AR3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AS3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AT3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AU3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AV3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AW3" s="3" t="inlineStr">
+      <c r="AV3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AW3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AX3" s="3" t="inlineStr">
+      <c r="AX3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="AY3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="AZ3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BA3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BB3" s="3" t="inlineStr">
+      <c r="AY3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="AZ3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BA3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BB3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="BC3" s="3" t="inlineStr">
+      <c r="BC3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="BD3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BE3" s="3" t="inlineStr">
+      <c r="BD3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BE3" s="4" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
       </c>
-      <c r="BF3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BG3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BH3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BI3" s="3" t="inlineStr">
-        <is>
-          <t>Char</t>
-        </is>
-      </c>
-      <c r="BJ3" s="3" t="inlineStr">
+      <c r="BF3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BG3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BH3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BI3" s="4" t="inlineStr">
+        <is>
+          <t>Char</t>
+        </is>
+      </c>
+      <c r="BJ3" s="4" t="inlineStr">
         <is>
           <t>Char</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="D4" s="3" t="n">
+      <c r="A4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="P4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="R4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="S4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="T4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="U4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="V4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="W4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="X4" s="3" t="n">
+      <c r="E4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="U4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="V4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="W4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="X4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="Y4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z4" s="3" t="n">
+      <c r="Y4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="Z4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="AA4" s="3" t="n">
+      <c r="AA4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="AB4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AC4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AD4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AE4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AF4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AG4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AH4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AI4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AJ4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AK4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AL4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AM4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AN4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AO4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AP4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AQ4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AR4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AS4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AT4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AU4" s="3" t="n">
+      <c r="AB4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AD4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AE4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AF4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AG4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AJ4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AM4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AN4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AO4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AP4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AQ4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AR4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AS4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AT4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AU4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="AV4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AW4" s="3" t="n">
+      <c r="AV4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AW4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="AX4" s="3" t="n">
+      <c r="AX4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="AY4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="AZ4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BA4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BB4" s="3" t="n">
+      <c r="AY4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="AZ4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BA4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BB4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="BC4" s="3" t="n">
+      <c r="BC4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="BD4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BE4" s="3" t="n">
+      <c r="BD4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BE4" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="BF4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BG4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BH4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BI4" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BJ4" s="3" t="n">
+      <c r="BF4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BG4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BH4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BI4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="BJ4" s="4" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>LB</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>S001</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>321</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="BI5" s="4" t="n"/>
-      <c r="BJ5" s="4" t="n"/>
+      <c r="BI5" s="5" t="str"/>
+      <c r="BJ5" s="5" t="str"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>CDISC-PILOT-01</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>LB</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>S002</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="BI6" s="4" t="n"/>
-      <c r="BJ6" s="4" t="n"/>
+      <c r="BI6" s="5" t="str"/>
+      <c r="BJ6" s="5" t="str"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>